<commit_message>
Update test_niveau_0_notation.xlsx - ajout colonnes completes
</commit_message>
<xml_diff>
--- a/test_niveau_0_notation.xlsx
+++ b/test_niveau_0_notation.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +58,14 @@
       <color rgb="00777777"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -91,8 +97,13 @@
         <fgColor rgb="00EEF5F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF2F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -142,11 +153,69 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="00267C7E"/>
+      </left>
+      <right style="medium">
+        <color rgb="00267C7E"/>
+      </right>
+      <top style="medium">
+        <color rgb="00267C7E"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00267C7E"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00267C7E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="00267C7E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00267C7E"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00267C7E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="00267C7E"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00267C7E"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -176,6 +245,26 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -543,19 +632,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -565,113 +658,151 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Saisir les points obtenus directement dans chaque colonne. La note finale /40 se calcule automatiquement. Seuil de réussite : 30/40</t>
+          <t>Erreur mineure = -0,25 pt  |  Erreur majeure = -0,50 pt  |  Saisie directe pour les autres exercices  |  Seuil de réussite : 30/40</t>
         </is>
       </c>
     </row>
     <row r="3" ht="6" customHeight="1"/>
-    <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Étudiant</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>LECTURE  /5</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="14" t="n"/>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>ÉCRITURE  /7</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="n"/>
+      <c r="G4" s="14" t="n"/>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>Alphabet /3</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>Solaire / Lunaire /10</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>Écriture attachée /4</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>Écriture détachée /4</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="inlineStr">
+        <is>
+          <t>Correction erreurs /7</t>
+        </is>
+      </c>
+      <c r="M4" s="12" t="inlineStr">
+        <is>
+          <t>NOTE FINALE /40</t>
+        </is>
+      </c>
+      <c r="N4" s="12" t="inlineStr">
+        <is>
+          <t>RÉSULTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Nom de l'étudiant</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>1. Alphabet
-/3</t>
+          <t>Err.
+min.</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>2. Vocal
-lecture
+          <t>Err.
+maj.</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>Note
 /5</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>3. Dictée
+          <t>Err.
+min.</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>Err.
+maj.</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>Note
 /7</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>4. Solaire /
-Lunaire
-/10</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>5. Écriture
-attachée
-/4</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>6. Écriture
-détachée
-/4</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>7. Correction
-erreurs
-/7</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>NOTE
-FINALE
-/40</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>RÉSULTAT</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="6">
-        <f>IF(COUNTA(A5)=0,"",SUM(B5,C5,D5,E5,F5,G5,H5))</f>
-        <v/>
-      </c>
-      <c r="J5" s="7">
-        <f>IF(I5="","",IF(I5&gt;=30,"✓ Admis","✗ Refusé"))</f>
-        <v/>
-      </c>
+      <c r="H5" s="15" t="inlineStr"/>
+      <c r="I5" s="15" t="inlineStr"/>
+      <c r="J5" s="15" t="inlineStr"/>
+      <c r="K5" s="15" t="inlineStr"/>
+      <c r="L5" s="15" t="inlineStr"/>
+      <c r="M5" s="15" t="inlineStr"/>
+      <c r="N5" s="15" t="inlineStr"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="8" t="n"/>
       <c r="B6" s="9" t="n"/>
       <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
+      <c r="D6" s="16">
+        <f>IF(OR(B6="",C6=""),"",MAX(0,5-B6*0.25-C6*0.5))</f>
+        <v/>
+      </c>
       <c r="E6" s="9" t="n"/>
       <c r="F6" s="9" t="n"/>
-      <c r="G6" s="9" t="n"/>
+      <c r="G6" s="16">
+        <f>IF(OR(E6="",F6=""),"",MAX(0,7-E6*0.25-F6*0.5))</f>
+        <v/>
+      </c>
       <c r="H6" s="9" t="n"/>
-      <c r="I6" s="6">
+      <c r="I6" s="9">
         <f>IF(COUNTA(A6)=0,"",SUM(B6,C6,D6,E6,F6,G6,H6))</f>
         <v/>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="9">
         <f>IF(I6="","",IF(I6&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K6" s="9" t="n"/>
+      <c r="L6" s="9" t="n"/>
+      <c r="M6" s="6">
+        <f>IF(COUNTA(A6)=0,"",IFERROR(SUM(D6,G6,H6,I6,J6,K6,L6),""))</f>
+        <v/>
+      </c>
+      <c r="N6" s="17">
+        <f>IF(M6="","",IF(M6&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -679,17 +810,33 @@
       <c r="A7" s="4" t="n"/>
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
+      <c r="D7" s="16">
+        <f>IF(OR(B7="",C7=""),"",MAX(0,5-B7*0.25-C7*0.5))</f>
+        <v/>
+      </c>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
+      <c r="G7" s="16">
+        <f>IF(OR(E7="",F7=""),"",MAX(0,7-E7*0.25-F7*0.5))</f>
+        <v/>
+      </c>
       <c r="H7" s="5" t="n"/>
-      <c r="I7" s="6">
+      <c r="I7" s="5">
         <f>IF(COUNTA(A7)=0,"",SUM(B7,C7,D7,E7,F7,G7,H7))</f>
         <v/>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="5">
         <f>IF(I7="","",IF(I7&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="6">
+        <f>IF(COUNTA(A7)=0,"",IFERROR(SUM(D7,G7,H7,I7,J7,K7,L7),""))</f>
+        <v/>
+      </c>
+      <c r="N7" s="18">
+        <f>IF(M7="","",IF(M7&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -697,17 +844,33 @@
       <c r="A8" s="8" t="n"/>
       <c r="B8" s="9" t="n"/>
       <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
+      <c r="D8" s="16">
+        <f>IF(OR(B8="",C8=""),"",MAX(0,5-B8*0.25-C8*0.5))</f>
+        <v/>
+      </c>
       <c r="E8" s="9" t="n"/>
       <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
+      <c r="G8" s="16">
+        <f>IF(OR(E8="",F8=""),"",MAX(0,7-E8*0.25-F8*0.5))</f>
+        <v/>
+      </c>
       <c r="H8" s="9" t="n"/>
-      <c r="I8" s="6">
+      <c r="I8" s="9">
         <f>IF(COUNTA(A8)=0,"",SUM(B8,C8,D8,E8,F8,G8,H8))</f>
         <v/>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="9">
         <f>IF(I8="","",IF(I8&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K8" s="9" t="n"/>
+      <c r="L8" s="9" t="n"/>
+      <c r="M8" s="6">
+        <f>IF(COUNTA(A8)=0,"",IFERROR(SUM(D8,G8,H8,I8,J8,K8,L8),""))</f>
+        <v/>
+      </c>
+      <c r="N8" s="17">
+        <f>IF(M8="","",IF(M8&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -715,17 +878,33 @@
       <c r="A9" s="4" t="n"/>
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
+      <c r="D9" s="16">
+        <f>IF(OR(B9="",C9=""),"",MAX(0,5-B9*0.25-C9*0.5))</f>
+        <v/>
+      </c>
       <c r="E9" s="5" t="n"/>
       <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
+      <c r="G9" s="16">
+        <f>IF(OR(E9="",F9=""),"",MAX(0,7-E9*0.25-F9*0.5))</f>
+        <v/>
+      </c>
       <c r="H9" s="5" t="n"/>
-      <c r="I9" s="6">
+      <c r="I9" s="5">
         <f>IF(COUNTA(A9)=0,"",SUM(B9,C9,D9,E9,F9,G9,H9))</f>
         <v/>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="5">
         <f>IF(I9="","",IF(I9&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K9" s="5" t="n"/>
+      <c r="L9" s="5" t="n"/>
+      <c r="M9" s="6">
+        <f>IF(COUNTA(A9)=0,"",IFERROR(SUM(D9,G9,H9,I9,J9,K9,L9),""))</f>
+        <v/>
+      </c>
+      <c r="N9" s="18">
+        <f>IF(M9="","",IF(M9&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -733,17 +912,33 @@
       <c r="A10" s="8" t="n"/>
       <c r="B10" s="9" t="n"/>
       <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
+      <c r="D10" s="16">
+        <f>IF(OR(B10="",C10=""),"",MAX(0,5-B10*0.25-C10*0.5))</f>
+        <v/>
+      </c>
       <c r="E10" s="9" t="n"/>
       <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9" t="n"/>
+      <c r="G10" s="16">
+        <f>IF(OR(E10="",F10=""),"",MAX(0,7-E10*0.25-F10*0.5))</f>
+        <v/>
+      </c>
       <c r="H10" s="9" t="n"/>
-      <c r="I10" s="6">
+      <c r="I10" s="9">
         <f>IF(COUNTA(A10)=0,"",SUM(B10,C10,D10,E10,F10,G10,H10))</f>
         <v/>
       </c>
-      <c r="J10" s="7">
+      <c r="J10" s="9">
         <f>IF(I10="","",IF(I10&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K10" s="9" t="n"/>
+      <c r="L10" s="9" t="n"/>
+      <c r="M10" s="6">
+        <f>IF(COUNTA(A10)=0,"",IFERROR(SUM(D10,G10,H10,I10,J10,K10,L10),""))</f>
+        <v/>
+      </c>
+      <c r="N10" s="17">
+        <f>IF(M10="","",IF(M10&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -751,17 +946,33 @@
       <c r="A11" s="4" t="n"/>
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
+      <c r="D11" s="16">
+        <f>IF(OR(B11="",C11=""),"",MAX(0,5-B11*0.25-C11*0.5))</f>
+        <v/>
+      </c>
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
+      <c r="G11" s="16">
+        <f>IF(OR(E11="",F11=""),"",MAX(0,7-E11*0.25-F11*0.5))</f>
+        <v/>
+      </c>
       <c r="H11" s="5" t="n"/>
-      <c r="I11" s="6">
+      <c r="I11" s="5">
         <f>IF(COUNTA(A11)=0,"",SUM(B11,C11,D11,E11,F11,G11,H11))</f>
         <v/>
       </c>
-      <c r="J11" s="7">
+      <c r="J11" s="5">
         <f>IF(I11="","",IF(I11&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K11" s="5" t="n"/>
+      <c r="L11" s="5" t="n"/>
+      <c r="M11" s="6">
+        <f>IF(COUNTA(A11)=0,"",IFERROR(SUM(D11,G11,H11,I11,J11,K11,L11),""))</f>
+        <v/>
+      </c>
+      <c r="N11" s="18">
+        <f>IF(M11="","",IF(M11&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -769,17 +980,33 @@
       <c r="A12" s="8" t="n"/>
       <c r="B12" s="9" t="n"/>
       <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
+      <c r="D12" s="16">
+        <f>IF(OR(B12="",C12=""),"",MAX(0,5-B12*0.25-C12*0.5))</f>
+        <v/>
+      </c>
       <c r="E12" s="9" t="n"/>
       <c r="F12" s="9" t="n"/>
-      <c r="G12" s="9" t="n"/>
+      <c r="G12" s="16">
+        <f>IF(OR(E12="",F12=""),"",MAX(0,7-E12*0.25-F12*0.5))</f>
+        <v/>
+      </c>
       <c r="H12" s="9" t="n"/>
-      <c r="I12" s="6">
+      <c r="I12" s="9">
         <f>IF(COUNTA(A12)=0,"",SUM(B12,C12,D12,E12,F12,G12,H12))</f>
         <v/>
       </c>
-      <c r="J12" s="7">
+      <c r="J12" s="9">
         <f>IF(I12="","",IF(I12&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K12" s="9" t="n"/>
+      <c r="L12" s="9" t="n"/>
+      <c r="M12" s="6">
+        <f>IF(COUNTA(A12)=0,"",IFERROR(SUM(D12,G12,H12,I12,J12,K12,L12),""))</f>
+        <v/>
+      </c>
+      <c r="N12" s="17">
+        <f>IF(M12="","",IF(M12&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -787,17 +1014,33 @@
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
+      <c r="D13" s="16">
+        <f>IF(OR(B13="",C13=""),"",MAX(0,5-B13*0.25-C13*0.5))</f>
+        <v/>
+      </c>
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
+      <c r="G13" s="16">
+        <f>IF(OR(E13="",F13=""),"",MAX(0,7-E13*0.25-F13*0.5))</f>
+        <v/>
+      </c>
       <c r="H13" s="5" t="n"/>
-      <c r="I13" s="6">
+      <c r="I13" s="5">
         <f>IF(COUNTA(A13)=0,"",SUM(B13,C13,D13,E13,F13,G13,H13))</f>
         <v/>
       </c>
-      <c r="J13" s="7">
+      <c r="J13" s="5">
         <f>IF(I13="","",IF(I13&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K13" s="5" t="n"/>
+      <c r="L13" s="5" t="n"/>
+      <c r="M13" s="6">
+        <f>IF(COUNTA(A13)=0,"",IFERROR(SUM(D13,G13,H13,I13,J13,K13,L13),""))</f>
+        <v/>
+      </c>
+      <c r="N13" s="18">
+        <f>IF(M13="","",IF(M13&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -805,17 +1048,33 @@
       <c r="A14" s="8" t="n"/>
       <c r="B14" s="9" t="n"/>
       <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
+      <c r="D14" s="16">
+        <f>IF(OR(B14="",C14=""),"",MAX(0,5-B14*0.25-C14*0.5))</f>
+        <v/>
+      </c>
       <c r="E14" s="9" t="n"/>
       <c r="F14" s="9" t="n"/>
-      <c r="G14" s="9" t="n"/>
+      <c r="G14" s="16">
+        <f>IF(OR(E14="",F14=""),"",MAX(0,7-E14*0.25-F14*0.5))</f>
+        <v/>
+      </c>
       <c r="H14" s="9" t="n"/>
-      <c r="I14" s="6">
+      <c r="I14" s="9">
         <f>IF(COUNTA(A14)=0,"",SUM(B14,C14,D14,E14,F14,G14,H14))</f>
         <v/>
       </c>
-      <c r="J14" s="7">
+      <c r="J14" s="9">
         <f>IF(I14="","",IF(I14&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K14" s="9" t="n"/>
+      <c r="L14" s="9" t="n"/>
+      <c r="M14" s="6">
+        <f>IF(COUNTA(A14)=0,"",IFERROR(SUM(D14,G14,H14,I14,J14,K14,L14),""))</f>
+        <v/>
+      </c>
+      <c r="N14" s="17">
+        <f>IF(M14="","",IF(M14&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -823,17 +1082,33 @@
       <c r="A15" s="4" t="n"/>
       <c r="B15" s="5" t="n"/>
       <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
+      <c r="D15" s="16">
+        <f>IF(OR(B15="",C15=""),"",MAX(0,5-B15*0.25-C15*0.5))</f>
+        <v/>
+      </c>
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
+      <c r="G15" s="16">
+        <f>IF(OR(E15="",F15=""),"",MAX(0,7-E15*0.25-F15*0.5))</f>
+        <v/>
+      </c>
       <c r="H15" s="5" t="n"/>
-      <c r="I15" s="6">
+      <c r="I15" s="5">
         <f>IF(COUNTA(A15)=0,"",SUM(B15,C15,D15,E15,F15,G15,H15))</f>
         <v/>
       </c>
-      <c r="J15" s="7">
+      <c r="J15" s="5">
         <f>IF(I15="","",IF(I15&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K15" s="5" t="n"/>
+      <c r="L15" s="5" t="n"/>
+      <c r="M15" s="6">
+        <f>IF(COUNTA(A15)=0,"",IFERROR(SUM(D15,G15,H15,I15,J15,K15,L15),""))</f>
+        <v/>
+      </c>
+      <c r="N15" s="18">
+        <f>IF(M15="","",IF(M15&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -841,17 +1116,33 @@
       <c r="A16" s="8" t="n"/>
       <c r="B16" s="9" t="n"/>
       <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9" t="n"/>
+      <c r="D16" s="16">
+        <f>IF(OR(B16="",C16=""),"",MAX(0,5-B16*0.25-C16*0.5))</f>
+        <v/>
+      </c>
       <c r="E16" s="9" t="n"/>
       <c r="F16" s="9" t="n"/>
-      <c r="G16" s="9" t="n"/>
+      <c r="G16" s="16">
+        <f>IF(OR(E16="",F16=""),"",MAX(0,7-E16*0.25-F16*0.5))</f>
+        <v/>
+      </c>
       <c r="H16" s="9" t="n"/>
-      <c r="I16" s="6">
+      <c r="I16" s="9">
         <f>IF(COUNTA(A16)=0,"",SUM(B16,C16,D16,E16,F16,G16,H16))</f>
         <v/>
       </c>
-      <c r="J16" s="7">
+      <c r="J16" s="9">
         <f>IF(I16="","",IF(I16&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K16" s="9" t="n"/>
+      <c r="L16" s="9" t="n"/>
+      <c r="M16" s="6">
+        <f>IF(COUNTA(A16)=0,"",IFERROR(SUM(D16,G16,H16,I16,J16,K16,L16),""))</f>
+        <v/>
+      </c>
+      <c r="N16" s="17">
+        <f>IF(M16="","",IF(M16&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -859,17 +1150,33 @@
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="5" t="n"/>
       <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
+      <c r="D17" s="16">
+        <f>IF(OR(B17="",C17=""),"",MAX(0,5-B17*0.25-C17*0.5))</f>
+        <v/>
+      </c>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
+      <c r="G17" s="16">
+        <f>IF(OR(E17="",F17=""),"",MAX(0,7-E17*0.25-F17*0.5))</f>
+        <v/>
+      </c>
       <c r="H17" s="5" t="n"/>
-      <c r="I17" s="6">
+      <c r="I17" s="5">
         <f>IF(COUNTA(A17)=0,"",SUM(B17,C17,D17,E17,F17,G17,H17))</f>
         <v/>
       </c>
-      <c r="J17" s="7">
+      <c r="J17" s="5">
         <f>IF(I17="","",IF(I17&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K17" s="5" t="n"/>
+      <c r="L17" s="5" t="n"/>
+      <c r="M17" s="6">
+        <f>IF(COUNTA(A17)=0,"",IFERROR(SUM(D17,G17,H17,I17,J17,K17,L17),""))</f>
+        <v/>
+      </c>
+      <c r="N17" s="18">
+        <f>IF(M17="","",IF(M17&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -877,17 +1184,33 @@
       <c r="A18" s="8" t="n"/>
       <c r="B18" s="9" t="n"/>
       <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
+      <c r="D18" s="16">
+        <f>IF(OR(B18="",C18=""),"",MAX(0,5-B18*0.25-C18*0.5))</f>
+        <v/>
+      </c>
       <c r="E18" s="9" t="n"/>
       <c r="F18" s="9" t="n"/>
-      <c r="G18" s="9" t="n"/>
+      <c r="G18" s="16">
+        <f>IF(OR(E18="",F18=""),"",MAX(0,7-E18*0.25-F18*0.5))</f>
+        <v/>
+      </c>
       <c r="H18" s="9" t="n"/>
-      <c r="I18" s="6">
+      <c r="I18" s="9">
         <f>IF(COUNTA(A18)=0,"",SUM(B18,C18,D18,E18,F18,G18,H18))</f>
         <v/>
       </c>
-      <c r="J18" s="7">
+      <c r="J18" s="9">
         <f>IF(I18="","",IF(I18&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K18" s="9" t="n"/>
+      <c r="L18" s="9" t="n"/>
+      <c r="M18" s="6">
+        <f>IF(COUNTA(A18)=0,"",IFERROR(SUM(D18,G18,H18,I18,J18,K18,L18),""))</f>
+        <v/>
+      </c>
+      <c r="N18" s="17">
+        <f>IF(M18="","",IF(M18&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -895,17 +1218,33 @@
       <c r="A19" s="4" t="n"/>
       <c r="B19" s="5" t="n"/>
       <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
+      <c r="D19" s="16">
+        <f>IF(OR(B19="",C19=""),"",MAX(0,5-B19*0.25-C19*0.5))</f>
+        <v/>
+      </c>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
+      <c r="G19" s="16">
+        <f>IF(OR(E19="",F19=""),"",MAX(0,7-E19*0.25-F19*0.5))</f>
+        <v/>
+      </c>
       <c r="H19" s="5" t="n"/>
-      <c r="I19" s="6">
+      <c r="I19" s="5">
         <f>IF(COUNTA(A19)=0,"",SUM(B19,C19,D19,E19,F19,G19,H19))</f>
         <v/>
       </c>
-      <c r="J19" s="7">
+      <c r="J19" s="5">
         <f>IF(I19="","",IF(I19&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K19" s="5" t="n"/>
+      <c r="L19" s="5" t="n"/>
+      <c r="M19" s="6">
+        <f>IF(COUNTA(A19)=0,"",IFERROR(SUM(D19,G19,H19,I19,J19,K19,L19),""))</f>
+        <v/>
+      </c>
+      <c r="N19" s="18">
+        <f>IF(M19="","",IF(M19&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -913,17 +1252,33 @@
       <c r="A20" s="8" t="n"/>
       <c r="B20" s="9" t="n"/>
       <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
+      <c r="D20" s="16">
+        <f>IF(OR(B20="",C20=""),"",MAX(0,5-B20*0.25-C20*0.5))</f>
+        <v/>
+      </c>
       <c r="E20" s="9" t="n"/>
       <c r="F20" s="9" t="n"/>
-      <c r="G20" s="9" t="n"/>
+      <c r="G20" s="16">
+        <f>IF(OR(E20="",F20=""),"",MAX(0,7-E20*0.25-F20*0.5))</f>
+        <v/>
+      </c>
       <c r="H20" s="9" t="n"/>
-      <c r="I20" s="6">
+      <c r="I20" s="9">
         <f>IF(COUNTA(A20)=0,"",SUM(B20,C20,D20,E20,F20,G20,H20))</f>
         <v/>
       </c>
-      <c r="J20" s="7">
+      <c r="J20" s="9">
         <f>IF(I20="","",IF(I20&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K20" s="9" t="n"/>
+      <c r="L20" s="9" t="n"/>
+      <c r="M20" s="6">
+        <f>IF(COUNTA(A20)=0,"",IFERROR(SUM(D20,G20,H20,I20,J20,K20,L20),""))</f>
+        <v/>
+      </c>
+      <c r="N20" s="17">
+        <f>IF(M20="","",IF(M20&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -931,17 +1286,33 @@
       <c r="A21" s="4" t="n"/>
       <c r="B21" s="5" t="n"/>
       <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
+      <c r="D21" s="16">
+        <f>IF(OR(B21="",C21=""),"",MAX(0,5-B21*0.25-C21*0.5))</f>
+        <v/>
+      </c>
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
+      <c r="G21" s="16">
+        <f>IF(OR(E21="",F21=""),"",MAX(0,7-E21*0.25-F21*0.5))</f>
+        <v/>
+      </c>
       <c r="H21" s="5" t="n"/>
-      <c r="I21" s="6">
+      <c r="I21" s="5">
         <f>IF(COUNTA(A21)=0,"",SUM(B21,C21,D21,E21,F21,G21,H21))</f>
         <v/>
       </c>
-      <c r="J21" s="7">
+      <c r="J21" s="5">
         <f>IF(I21="","",IF(I21&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K21" s="5" t="n"/>
+      <c r="L21" s="5" t="n"/>
+      <c r="M21" s="6">
+        <f>IF(COUNTA(A21)=0,"",IFERROR(SUM(D21,G21,H21,I21,J21,K21,L21),""))</f>
+        <v/>
+      </c>
+      <c r="N21" s="18">
+        <f>IF(M21="","",IF(M21&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -949,17 +1320,33 @@
       <c r="A22" s="8" t="n"/>
       <c r="B22" s="9" t="n"/>
       <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
+      <c r="D22" s="16">
+        <f>IF(OR(B22="",C22=""),"",MAX(0,5-B22*0.25-C22*0.5))</f>
+        <v/>
+      </c>
       <c r="E22" s="9" t="n"/>
       <c r="F22" s="9" t="n"/>
-      <c r="G22" s="9" t="n"/>
+      <c r="G22" s="16">
+        <f>IF(OR(E22="",F22=""),"",MAX(0,7-E22*0.25-F22*0.5))</f>
+        <v/>
+      </c>
       <c r="H22" s="9" t="n"/>
-      <c r="I22" s="6">
+      <c r="I22" s="9">
         <f>IF(COUNTA(A22)=0,"",SUM(B22,C22,D22,E22,F22,G22,H22))</f>
         <v/>
       </c>
-      <c r="J22" s="7">
+      <c r="J22" s="9">
         <f>IF(I22="","",IF(I22&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K22" s="9" t="n"/>
+      <c r="L22" s="9" t="n"/>
+      <c r="M22" s="6">
+        <f>IF(COUNTA(A22)=0,"",IFERROR(SUM(D22,G22,H22,I22,J22,K22,L22),""))</f>
+        <v/>
+      </c>
+      <c r="N22" s="17">
+        <f>IF(M22="","",IF(M22&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -967,17 +1354,33 @@
       <c r="A23" s="4" t="n"/>
       <c r="B23" s="5" t="n"/>
       <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
+      <c r="D23" s="16">
+        <f>IF(OR(B23="",C23=""),"",MAX(0,5-B23*0.25-C23*0.5))</f>
+        <v/>
+      </c>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
+      <c r="G23" s="16">
+        <f>IF(OR(E23="",F23=""),"",MAX(0,7-E23*0.25-F23*0.5))</f>
+        <v/>
+      </c>
       <c r="H23" s="5" t="n"/>
-      <c r="I23" s="6">
+      <c r="I23" s="5">
         <f>IF(COUNTA(A23)=0,"",SUM(B23,C23,D23,E23,F23,G23,H23))</f>
         <v/>
       </c>
-      <c r="J23" s="7">
+      <c r="J23" s="5">
         <f>IF(I23="","",IF(I23&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K23" s="5" t="n"/>
+      <c r="L23" s="5" t="n"/>
+      <c r="M23" s="6">
+        <f>IF(COUNTA(A23)=0,"",IFERROR(SUM(D23,G23,H23,I23,J23,K23,L23),""))</f>
+        <v/>
+      </c>
+      <c r="N23" s="18">
+        <f>IF(M23="","",IF(M23&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -985,17 +1388,33 @@
       <c r="A24" s="8" t="n"/>
       <c r="B24" s="9" t="n"/>
       <c r="C24" s="9" t="n"/>
-      <c r="D24" s="9" t="n"/>
+      <c r="D24" s="16">
+        <f>IF(OR(B24="",C24=""),"",MAX(0,5-B24*0.25-C24*0.5))</f>
+        <v/>
+      </c>
       <c r="E24" s="9" t="n"/>
       <c r="F24" s="9" t="n"/>
-      <c r="G24" s="9" t="n"/>
+      <c r="G24" s="16">
+        <f>IF(OR(E24="",F24=""),"",MAX(0,7-E24*0.25-F24*0.5))</f>
+        <v/>
+      </c>
       <c r="H24" s="9" t="n"/>
-      <c r="I24" s="6">
+      <c r="I24" s="9">
         <f>IF(COUNTA(A24)=0,"",SUM(B24,C24,D24,E24,F24,G24,H24))</f>
         <v/>
       </c>
-      <c r="J24" s="7">
+      <c r="J24" s="9">
         <f>IF(I24="","",IF(I24&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K24" s="9" t="n"/>
+      <c r="L24" s="9" t="n"/>
+      <c r="M24" s="6">
+        <f>IF(COUNTA(A24)=0,"",IFERROR(SUM(D24,G24,H24,I24,J24,K24,L24),""))</f>
+        <v/>
+      </c>
+      <c r="N24" s="17">
+        <f>IF(M24="","",IF(M24&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1003,17 +1422,33 @@
       <c r="A25" s="4" t="n"/>
       <c r="B25" s="5" t="n"/>
       <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
+      <c r="D25" s="16">
+        <f>IF(OR(B25="",C25=""),"",MAX(0,5-B25*0.25-C25*0.5))</f>
+        <v/>
+      </c>
       <c r="E25" s="5" t="n"/>
       <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
+      <c r="G25" s="16">
+        <f>IF(OR(E25="",F25=""),"",MAX(0,7-E25*0.25-F25*0.5))</f>
+        <v/>
+      </c>
       <c r="H25" s="5" t="n"/>
-      <c r="I25" s="6">
+      <c r="I25" s="5">
         <f>IF(COUNTA(A25)=0,"",SUM(B25,C25,D25,E25,F25,G25,H25))</f>
         <v/>
       </c>
-      <c r="J25" s="7">
+      <c r="J25" s="5">
         <f>IF(I25="","",IF(I25&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K25" s="5" t="n"/>
+      <c r="L25" s="5" t="n"/>
+      <c r="M25" s="6">
+        <f>IF(COUNTA(A25)=0,"",IFERROR(SUM(D25,G25,H25,I25,J25,K25,L25),""))</f>
+        <v/>
+      </c>
+      <c r="N25" s="18">
+        <f>IF(M25="","",IF(M25&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1021,17 +1456,33 @@
       <c r="A26" s="8" t="n"/>
       <c r="B26" s="9" t="n"/>
       <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
+      <c r="D26" s="16">
+        <f>IF(OR(B26="",C26=""),"",MAX(0,5-B26*0.25-C26*0.5))</f>
+        <v/>
+      </c>
       <c r="E26" s="9" t="n"/>
       <c r="F26" s="9" t="n"/>
-      <c r="G26" s="9" t="n"/>
+      <c r="G26" s="16">
+        <f>IF(OR(E26="",F26=""),"",MAX(0,7-E26*0.25-F26*0.5))</f>
+        <v/>
+      </c>
       <c r="H26" s="9" t="n"/>
-      <c r="I26" s="6">
+      <c r="I26" s="9">
         <f>IF(COUNTA(A26)=0,"",SUM(B26,C26,D26,E26,F26,G26,H26))</f>
         <v/>
       </c>
-      <c r="J26" s="7">
+      <c r="J26" s="9">
         <f>IF(I26="","",IF(I26&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K26" s="9" t="n"/>
+      <c r="L26" s="9" t="n"/>
+      <c r="M26" s="6">
+        <f>IF(COUNTA(A26)=0,"",IFERROR(SUM(D26,G26,H26,I26,J26,K26,L26),""))</f>
+        <v/>
+      </c>
+      <c r="N26" s="17">
+        <f>IF(M26="","",IF(M26&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1039,17 +1490,33 @@
       <c r="A27" s="4" t="n"/>
       <c r="B27" s="5" t="n"/>
       <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
+      <c r="D27" s="16">
+        <f>IF(OR(B27="",C27=""),"",MAX(0,5-B27*0.25-C27*0.5))</f>
+        <v/>
+      </c>
       <c r="E27" s="5" t="n"/>
       <c r="F27" s="5" t="n"/>
-      <c r="G27" s="5" t="n"/>
+      <c r="G27" s="16">
+        <f>IF(OR(E27="",F27=""),"",MAX(0,7-E27*0.25-F27*0.5))</f>
+        <v/>
+      </c>
       <c r="H27" s="5" t="n"/>
-      <c r="I27" s="6">
+      <c r="I27" s="5">
         <f>IF(COUNTA(A27)=0,"",SUM(B27,C27,D27,E27,F27,G27,H27))</f>
         <v/>
       </c>
-      <c r="J27" s="7">
+      <c r="J27" s="5">
         <f>IF(I27="","",IF(I27&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K27" s="5" t="n"/>
+      <c r="L27" s="5" t="n"/>
+      <c r="M27" s="6">
+        <f>IF(COUNTA(A27)=0,"",IFERROR(SUM(D27,G27,H27,I27,J27,K27,L27),""))</f>
+        <v/>
+      </c>
+      <c r="N27" s="18">
+        <f>IF(M27="","",IF(M27&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1057,17 +1524,33 @@
       <c r="A28" s="8" t="n"/>
       <c r="B28" s="9" t="n"/>
       <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
+      <c r="D28" s="16">
+        <f>IF(OR(B28="",C28=""),"",MAX(0,5-B28*0.25-C28*0.5))</f>
+        <v/>
+      </c>
       <c r="E28" s="9" t="n"/>
       <c r="F28" s="9" t="n"/>
-      <c r="G28" s="9" t="n"/>
+      <c r="G28" s="16">
+        <f>IF(OR(E28="",F28=""),"",MAX(0,7-E28*0.25-F28*0.5))</f>
+        <v/>
+      </c>
       <c r="H28" s="9" t="n"/>
-      <c r="I28" s="6">
+      <c r="I28" s="9">
         <f>IF(COUNTA(A28)=0,"",SUM(B28,C28,D28,E28,F28,G28,H28))</f>
         <v/>
       </c>
-      <c r="J28" s="7">
+      <c r="J28" s="9">
         <f>IF(I28="","",IF(I28&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K28" s="9" t="n"/>
+      <c r="L28" s="9" t="n"/>
+      <c r="M28" s="6">
+        <f>IF(COUNTA(A28)=0,"",IFERROR(SUM(D28,G28,H28,I28,J28,K28,L28),""))</f>
+        <v/>
+      </c>
+      <c r="N28" s="17">
+        <f>IF(M28="","",IF(M28&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1075,17 +1558,33 @@
       <c r="A29" s="4" t="n"/>
       <c r="B29" s="5" t="n"/>
       <c r="C29" s="5" t="n"/>
-      <c r="D29" s="5" t="n"/>
+      <c r="D29" s="16">
+        <f>IF(OR(B29="",C29=""),"",MAX(0,5-B29*0.25-C29*0.5))</f>
+        <v/>
+      </c>
       <c r="E29" s="5" t="n"/>
       <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
+      <c r="G29" s="16">
+        <f>IF(OR(E29="",F29=""),"",MAX(0,7-E29*0.25-F29*0.5))</f>
+        <v/>
+      </c>
       <c r="H29" s="5" t="n"/>
-      <c r="I29" s="6">
+      <c r="I29" s="5">
         <f>IF(COUNTA(A29)=0,"",SUM(B29,C29,D29,E29,F29,G29,H29))</f>
         <v/>
       </c>
-      <c r="J29" s="7">
+      <c r="J29" s="5">
         <f>IF(I29="","",IF(I29&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K29" s="5" t="n"/>
+      <c r="L29" s="5" t="n"/>
+      <c r="M29" s="6">
+        <f>IF(COUNTA(A29)=0,"",IFERROR(SUM(D29,G29,H29,I29,J29,K29,L29),""))</f>
+        <v/>
+      </c>
+      <c r="N29" s="18">
+        <f>IF(M29="","",IF(M29&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1093,17 +1592,33 @@
       <c r="A30" s="8" t="n"/>
       <c r="B30" s="9" t="n"/>
       <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
+      <c r="D30" s="16">
+        <f>IF(OR(B30="",C30=""),"",MAX(0,5-B30*0.25-C30*0.5))</f>
+        <v/>
+      </c>
       <c r="E30" s="9" t="n"/>
       <c r="F30" s="9" t="n"/>
-      <c r="G30" s="9" t="n"/>
+      <c r="G30" s="16">
+        <f>IF(OR(E30="",F30=""),"",MAX(0,7-E30*0.25-F30*0.5))</f>
+        <v/>
+      </c>
       <c r="H30" s="9" t="n"/>
-      <c r="I30" s="6">
+      <c r="I30" s="9">
         <f>IF(COUNTA(A30)=0,"",SUM(B30,C30,D30,E30,F30,G30,H30))</f>
         <v/>
       </c>
-      <c r="J30" s="7">
+      <c r="J30" s="9">
         <f>IF(I30="","",IF(I30&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K30" s="9" t="n"/>
+      <c r="L30" s="9" t="n"/>
+      <c r="M30" s="6">
+        <f>IF(COUNTA(A30)=0,"",IFERROR(SUM(D30,G30,H30,I30,J30,K30,L30),""))</f>
+        <v/>
+      </c>
+      <c r="N30" s="17">
+        <f>IF(M30="","",IF(M30&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1111,17 +1626,33 @@
       <c r="A31" s="4" t="n"/>
       <c r="B31" s="5" t="n"/>
       <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
+      <c r="D31" s="16">
+        <f>IF(OR(B31="",C31=""),"",MAX(0,5-B31*0.25-C31*0.5))</f>
+        <v/>
+      </c>
       <c r="E31" s="5" t="n"/>
       <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
+      <c r="G31" s="16">
+        <f>IF(OR(E31="",F31=""),"",MAX(0,7-E31*0.25-F31*0.5))</f>
+        <v/>
+      </c>
       <c r="H31" s="5" t="n"/>
-      <c r="I31" s="6">
+      <c r="I31" s="5">
         <f>IF(COUNTA(A31)=0,"",SUM(B31,C31,D31,E31,F31,G31,H31))</f>
         <v/>
       </c>
-      <c r="J31" s="7">
+      <c r="J31" s="5">
         <f>IF(I31="","",IF(I31&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K31" s="5" t="n"/>
+      <c r="L31" s="5" t="n"/>
+      <c r="M31" s="6">
+        <f>IF(COUNTA(A31)=0,"",IFERROR(SUM(D31,G31,H31,I31,J31,K31,L31),""))</f>
+        <v/>
+      </c>
+      <c r="N31" s="18">
+        <f>IF(M31="","",IF(M31&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1129,17 +1660,33 @@
       <c r="A32" s="8" t="n"/>
       <c r="B32" s="9" t="n"/>
       <c r="C32" s="9" t="n"/>
-      <c r="D32" s="9" t="n"/>
+      <c r="D32" s="16">
+        <f>IF(OR(B32="",C32=""),"",MAX(0,5-B32*0.25-C32*0.5))</f>
+        <v/>
+      </c>
       <c r="E32" s="9" t="n"/>
       <c r="F32" s="9" t="n"/>
-      <c r="G32" s="9" t="n"/>
+      <c r="G32" s="16">
+        <f>IF(OR(E32="",F32=""),"",MAX(0,7-E32*0.25-F32*0.5))</f>
+        <v/>
+      </c>
       <c r="H32" s="9" t="n"/>
-      <c r="I32" s="6">
+      <c r="I32" s="9">
         <f>IF(COUNTA(A32)=0,"",SUM(B32,C32,D32,E32,F32,G32,H32))</f>
         <v/>
       </c>
-      <c r="J32" s="7">
+      <c r="J32" s="9">
         <f>IF(I32="","",IF(I32&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K32" s="9" t="n"/>
+      <c r="L32" s="9" t="n"/>
+      <c r="M32" s="6">
+        <f>IF(COUNTA(A32)=0,"",IFERROR(SUM(D32,G32,H32,I32,J32,K32,L32),""))</f>
+        <v/>
+      </c>
+      <c r="N32" s="17">
+        <f>IF(M32="","",IF(M32&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1147,17 +1694,33 @@
       <c r="A33" s="4" t="n"/>
       <c r="B33" s="5" t="n"/>
       <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
+      <c r="D33" s="16">
+        <f>IF(OR(B33="",C33=""),"",MAX(0,5-B33*0.25-C33*0.5))</f>
+        <v/>
+      </c>
       <c r="E33" s="5" t="n"/>
       <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
+      <c r="G33" s="16">
+        <f>IF(OR(E33="",F33=""),"",MAX(0,7-E33*0.25-F33*0.5))</f>
+        <v/>
+      </c>
       <c r="H33" s="5" t="n"/>
-      <c r="I33" s="6">
+      <c r="I33" s="5">
         <f>IF(COUNTA(A33)=0,"",SUM(B33,C33,D33,E33,F33,G33,H33))</f>
         <v/>
       </c>
-      <c r="J33" s="7">
+      <c r="J33" s="5">
         <f>IF(I33="","",IF(I33&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K33" s="5" t="n"/>
+      <c r="L33" s="5" t="n"/>
+      <c r="M33" s="6">
+        <f>IF(COUNTA(A33)=0,"",IFERROR(SUM(D33,G33,H33,I33,J33,K33,L33),""))</f>
+        <v/>
+      </c>
+      <c r="N33" s="18">
+        <f>IF(M33="","",IF(M33&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1165,17 +1728,33 @@
       <c r="A34" s="8" t="n"/>
       <c r="B34" s="9" t="n"/>
       <c r="C34" s="9" t="n"/>
-      <c r="D34" s="9" t="n"/>
+      <c r="D34" s="16">
+        <f>IF(OR(B34="",C34=""),"",MAX(0,5-B34*0.25-C34*0.5))</f>
+        <v/>
+      </c>
       <c r="E34" s="9" t="n"/>
       <c r="F34" s="9" t="n"/>
-      <c r="G34" s="9" t="n"/>
+      <c r="G34" s="16">
+        <f>IF(OR(E34="",F34=""),"",MAX(0,7-E34*0.25-F34*0.5))</f>
+        <v/>
+      </c>
       <c r="H34" s="9" t="n"/>
-      <c r="I34" s="6">
+      <c r="I34" s="9">
         <f>IF(COUNTA(A34)=0,"",SUM(B34,C34,D34,E34,F34,G34,H34))</f>
         <v/>
       </c>
-      <c r="J34" s="7">
+      <c r="J34" s="9">
         <f>IF(I34="","",IF(I34&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K34" s="9" t="n"/>
+      <c r="L34" s="9" t="n"/>
+      <c r="M34" s="6">
+        <f>IF(COUNTA(A34)=0,"",IFERROR(SUM(D34,G34,H34,I34,J34,K34,L34),""))</f>
+        <v/>
+      </c>
+      <c r="N34" s="17">
+        <f>IF(M34="","",IF(M34&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1183,17 +1762,33 @@
       <c r="A35" s="4" t="n"/>
       <c r="B35" s="5" t="n"/>
       <c r="C35" s="5" t="n"/>
-      <c r="D35" s="5" t="n"/>
+      <c r="D35" s="16">
+        <f>IF(OR(B35="",C35=""),"",MAX(0,5-B35*0.25-C35*0.5))</f>
+        <v/>
+      </c>
       <c r="E35" s="5" t="n"/>
       <c r="F35" s="5" t="n"/>
-      <c r="G35" s="5" t="n"/>
+      <c r="G35" s="16">
+        <f>IF(OR(E35="",F35=""),"",MAX(0,7-E35*0.25-F35*0.5))</f>
+        <v/>
+      </c>
       <c r="H35" s="5" t="n"/>
-      <c r="I35" s="6">
+      <c r="I35" s="5">
         <f>IF(COUNTA(A35)=0,"",SUM(B35,C35,D35,E35,F35,G35,H35))</f>
         <v/>
       </c>
-      <c r="J35" s="7">
+      <c r="J35" s="5">
         <f>IF(I35="","",IF(I35&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K35" s="5" t="n"/>
+      <c r="L35" s="5" t="n"/>
+      <c r="M35" s="6">
+        <f>IF(COUNTA(A35)=0,"",IFERROR(SUM(D35,G35,H35,I35,J35,K35,L35),""))</f>
+        <v/>
+      </c>
+      <c r="N35" s="18">
+        <f>IF(M35="","",IF(M35&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1201,17 +1796,33 @@
       <c r="A36" s="8" t="n"/>
       <c r="B36" s="9" t="n"/>
       <c r="C36" s="9" t="n"/>
-      <c r="D36" s="9" t="n"/>
+      <c r="D36" s="16">
+        <f>IF(OR(B36="",C36=""),"",MAX(0,5-B36*0.25-C36*0.5))</f>
+        <v/>
+      </c>
       <c r="E36" s="9" t="n"/>
       <c r="F36" s="9" t="n"/>
-      <c r="G36" s="9" t="n"/>
+      <c r="G36" s="16">
+        <f>IF(OR(E36="",F36=""),"",MAX(0,7-E36*0.25-F36*0.5))</f>
+        <v/>
+      </c>
       <c r="H36" s="9" t="n"/>
-      <c r="I36" s="6">
+      <c r="I36" s="9">
         <f>IF(COUNTA(A36)=0,"",SUM(B36,C36,D36,E36,F36,G36,H36))</f>
         <v/>
       </c>
-      <c r="J36" s="7">
+      <c r="J36" s="9">
         <f>IF(I36="","",IF(I36&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K36" s="9" t="n"/>
+      <c r="L36" s="9" t="n"/>
+      <c r="M36" s="6">
+        <f>IF(COUNTA(A36)=0,"",IFERROR(SUM(D36,G36,H36,I36,J36,K36,L36),""))</f>
+        <v/>
+      </c>
+      <c r="N36" s="17">
+        <f>IF(M36="","",IF(M36&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1219,17 +1830,33 @@
       <c r="A37" s="4" t="n"/>
       <c r="B37" s="5" t="n"/>
       <c r="C37" s="5" t="n"/>
-      <c r="D37" s="5" t="n"/>
+      <c r="D37" s="16">
+        <f>IF(OR(B37="",C37=""),"",MAX(0,5-B37*0.25-C37*0.5))</f>
+        <v/>
+      </c>
       <c r="E37" s="5" t="n"/>
       <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
+      <c r="G37" s="16">
+        <f>IF(OR(E37="",F37=""),"",MAX(0,7-E37*0.25-F37*0.5))</f>
+        <v/>
+      </c>
       <c r="H37" s="5" t="n"/>
-      <c r="I37" s="6">
+      <c r="I37" s="5">
         <f>IF(COUNTA(A37)=0,"",SUM(B37,C37,D37,E37,F37,G37,H37))</f>
         <v/>
       </c>
-      <c r="J37" s="7">
+      <c r="J37" s="5">
         <f>IF(I37="","",IF(I37&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K37" s="5" t="n"/>
+      <c r="L37" s="5" t="n"/>
+      <c r="M37" s="6">
+        <f>IF(COUNTA(A37)=0,"",IFERROR(SUM(D37,G37,H37,I37,J37,K37,L37),""))</f>
+        <v/>
+      </c>
+      <c r="N37" s="18">
+        <f>IF(M37="","",IF(M37&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1237,17 +1864,33 @@
       <c r="A38" s="8" t="n"/>
       <c r="B38" s="9" t="n"/>
       <c r="C38" s="9" t="n"/>
-      <c r="D38" s="9" t="n"/>
+      <c r="D38" s="16">
+        <f>IF(OR(B38="",C38=""),"",MAX(0,5-B38*0.25-C38*0.5))</f>
+        <v/>
+      </c>
       <c r="E38" s="9" t="n"/>
       <c r="F38" s="9" t="n"/>
-      <c r="G38" s="9" t="n"/>
+      <c r="G38" s="16">
+        <f>IF(OR(E38="",F38=""),"",MAX(0,7-E38*0.25-F38*0.5))</f>
+        <v/>
+      </c>
       <c r="H38" s="9" t="n"/>
-      <c r="I38" s="6">
+      <c r="I38" s="9">
         <f>IF(COUNTA(A38)=0,"",SUM(B38,C38,D38,E38,F38,G38,H38))</f>
         <v/>
       </c>
-      <c r="J38" s="7">
+      <c r="J38" s="9">
         <f>IF(I38="","",IF(I38&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K38" s="9" t="n"/>
+      <c r="L38" s="9" t="n"/>
+      <c r="M38" s="6">
+        <f>IF(COUNTA(A38)=0,"",IFERROR(SUM(D38,G38,H38,I38,J38,K38,L38),""))</f>
+        <v/>
+      </c>
+      <c r="N38" s="17">
+        <f>IF(M38="","",IF(M38&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1255,17 +1898,33 @@
       <c r="A39" s="4" t="n"/>
       <c r="B39" s="5" t="n"/>
       <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="n"/>
+      <c r="D39" s="16">
+        <f>IF(OR(B39="",C39=""),"",MAX(0,5-B39*0.25-C39*0.5))</f>
+        <v/>
+      </c>
       <c r="E39" s="5" t="n"/>
       <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
+      <c r="G39" s="16">
+        <f>IF(OR(E39="",F39=""),"",MAX(0,7-E39*0.25-F39*0.5))</f>
+        <v/>
+      </c>
       <c r="H39" s="5" t="n"/>
-      <c r="I39" s="6">
+      <c r="I39" s="5">
         <f>IF(COUNTA(A39)=0,"",SUM(B39,C39,D39,E39,F39,G39,H39))</f>
         <v/>
       </c>
-      <c r="J39" s="7">
+      <c r="J39" s="5">
         <f>IF(I39="","",IF(I39&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K39" s="5" t="n"/>
+      <c r="L39" s="5" t="n"/>
+      <c r="M39" s="6">
+        <f>IF(COUNTA(A39)=0,"",IFERROR(SUM(D39,G39,H39,I39,J39,K39,L39),""))</f>
+        <v/>
+      </c>
+      <c r="N39" s="18">
+        <f>IF(M39="","",IF(M39&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1273,17 +1932,33 @@
       <c r="A40" s="8" t="n"/>
       <c r="B40" s="9" t="n"/>
       <c r="C40" s="9" t="n"/>
-      <c r="D40" s="9" t="n"/>
+      <c r="D40" s="16">
+        <f>IF(OR(B40="",C40=""),"",MAX(0,5-B40*0.25-C40*0.5))</f>
+        <v/>
+      </c>
       <c r="E40" s="9" t="n"/>
       <c r="F40" s="9" t="n"/>
-      <c r="G40" s="9" t="n"/>
+      <c r="G40" s="16">
+        <f>IF(OR(E40="",F40=""),"",MAX(0,7-E40*0.25-F40*0.5))</f>
+        <v/>
+      </c>
       <c r="H40" s="9" t="n"/>
-      <c r="I40" s="6">
+      <c r="I40" s="9">
         <f>IF(COUNTA(A40)=0,"",SUM(B40,C40,D40,E40,F40,G40,H40))</f>
         <v/>
       </c>
-      <c r="J40" s="7">
+      <c r="J40" s="9">
         <f>IF(I40="","",IF(I40&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K40" s="9" t="n"/>
+      <c r="L40" s="9" t="n"/>
+      <c r="M40" s="6">
+        <f>IF(COUNTA(A40)=0,"",IFERROR(SUM(D40,G40,H40,I40,J40,K40,L40),""))</f>
+        <v/>
+      </c>
+      <c r="N40" s="17">
+        <f>IF(M40="","",IF(M40&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1291,17 +1966,33 @@
       <c r="A41" s="4" t="n"/>
       <c r="B41" s="5" t="n"/>
       <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
+      <c r="D41" s="16">
+        <f>IF(OR(B41="",C41=""),"",MAX(0,5-B41*0.25-C41*0.5))</f>
+        <v/>
+      </c>
       <c r="E41" s="5" t="n"/>
       <c r="F41" s="5" t="n"/>
-      <c r="G41" s="5" t="n"/>
+      <c r="G41" s="16">
+        <f>IF(OR(E41="",F41=""),"",MAX(0,7-E41*0.25-F41*0.5))</f>
+        <v/>
+      </c>
       <c r="H41" s="5" t="n"/>
-      <c r="I41" s="6">
+      <c r="I41" s="5">
         <f>IF(COUNTA(A41)=0,"",SUM(B41,C41,D41,E41,F41,G41,H41))</f>
         <v/>
       </c>
-      <c r="J41" s="7">
+      <c r="J41" s="5">
         <f>IF(I41="","",IF(I41&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K41" s="5" t="n"/>
+      <c r="L41" s="5" t="n"/>
+      <c r="M41" s="6">
+        <f>IF(COUNTA(A41)=0,"",IFERROR(SUM(D41,G41,H41,I41,J41,K41,L41),""))</f>
+        <v/>
+      </c>
+      <c r="N41" s="18">
+        <f>IF(M41="","",IF(M41&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1309,17 +2000,33 @@
       <c r="A42" s="8" t="n"/>
       <c r="B42" s="9" t="n"/>
       <c r="C42" s="9" t="n"/>
-      <c r="D42" s="9" t="n"/>
+      <c r="D42" s="16">
+        <f>IF(OR(B42="",C42=""),"",MAX(0,5-B42*0.25-C42*0.5))</f>
+        <v/>
+      </c>
       <c r="E42" s="9" t="n"/>
       <c r="F42" s="9" t="n"/>
-      <c r="G42" s="9" t="n"/>
+      <c r="G42" s="16">
+        <f>IF(OR(E42="",F42=""),"",MAX(0,7-E42*0.25-F42*0.5))</f>
+        <v/>
+      </c>
       <c r="H42" s="9" t="n"/>
-      <c r="I42" s="6">
+      <c r="I42" s="9">
         <f>IF(COUNTA(A42)=0,"",SUM(B42,C42,D42,E42,F42,G42,H42))</f>
         <v/>
       </c>
-      <c r="J42" s="7">
+      <c r="J42" s="9">
         <f>IF(I42="","",IF(I42&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K42" s="9" t="n"/>
+      <c r="L42" s="9" t="n"/>
+      <c r="M42" s="6">
+        <f>IF(COUNTA(A42)=0,"",IFERROR(SUM(D42,G42,H42,I42,J42,K42,L42),""))</f>
+        <v/>
+      </c>
+      <c r="N42" s="17">
+        <f>IF(M42="","",IF(M42&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1327,17 +2034,33 @@
       <c r="A43" s="4" t="n"/>
       <c r="B43" s="5" t="n"/>
       <c r="C43" s="5" t="n"/>
-      <c r="D43" s="5" t="n"/>
+      <c r="D43" s="16">
+        <f>IF(OR(B43="",C43=""),"",MAX(0,5-B43*0.25-C43*0.5))</f>
+        <v/>
+      </c>
       <c r="E43" s="5" t="n"/>
       <c r="F43" s="5" t="n"/>
-      <c r="G43" s="5" t="n"/>
+      <c r="G43" s="16">
+        <f>IF(OR(E43="",F43=""),"",MAX(0,7-E43*0.25-F43*0.5))</f>
+        <v/>
+      </c>
       <c r="H43" s="5" t="n"/>
-      <c r="I43" s="6">
+      <c r="I43" s="5">
         <f>IF(COUNTA(A43)=0,"",SUM(B43,C43,D43,E43,F43,G43,H43))</f>
         <v/>
       </c>
-      <c r="J43" s="7">
+      <c r="J43" s="5">
         <f>IF(I43="","",IF(I43&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K43" s="5" t="n"/>
+      <c r="L43" s="5" t="n"/>
+      <c r="M43" s="6">
+        <f>IF(COUNTA(A43)=0,"",IFERROR(SUM(D43,G43,H43,I43,J43,K43,L43),""))</f>
+        <v/>
+      </c>
+      <c r="N43" s="18">
+        <f>IF(M43="","",IF(M43&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1345,17 +2068,33 @@
       <c r="A44" s="8" t="n"/>
       <c r="B44" s="9" t="n"/>
       <c r="C44" s="9" t="n"/>
-      <c r="D44" s="9" t="n"/>
+      <c r="D44" s="16">
+        <f>IF(OR(B44="",C44=""),"",MAX(0,5-B44*0.25-C44*0.5))</f>
+        <v/>
+      </c>
       <c r="E44" s="9" t="n"/>
       <c r="F44" s="9" t="n"/>
-      <c r="G44" s="9" t="n"/>
+      <c r="G44" s="16">
+        <f>IF(OR(E44="",F44=""),"",MAX(0,7-E44*0.25-F44*0.5))</f>
+        <v/>
+      </c>
       <c r="H44" s="9" t="n"/>
-      <c r="I44" s="6">
+      <c r="I44" s="9">
         <f>IF(COUNTA(A44)=0,"",SUM(B44,C44,D44,E44,F44,G44,H44))</f>
         <v/>
       </c>
-      <c r="J44" s="7">
+      <c r="J44" s="9">
         <f>IF(I44="","",IF(I44&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K44" s="9" t="n"/>
+      <c r="L44" s="9" t="n"/>
+      <c r="M44" s="6">
+        <f>IF(COUNTA(A44)=0,"",IFERROR(SUM(D44,G44,H44,I44,J44,K44,L44),""))</f>
+        <v/>
+      </c>
+      <c r="N44" s="17">
+        <f>IF(M44="","",IF(M44&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1363,17 +2102,33 @@
       <c r="A45" s="4" t="n"/>
       <c r="B45" s="5" t="n"/>
       <c r="C45" s="5" t="n"/>
-      <c r="D45" s="5" t="n"/>
+      <c r="D45" s="16">
+        <f>IF(OR(B45="",C45=""),"",MAX(0,5-B45*0.25-C45*0.5))</f>
+        <v/>
+      </c>
       <c r="E45" s="5" t="n"/>
       <c r="F45" s="5" t="n"/>
-      <c r="G45" s="5" t="n"/>
+      <c r="G45" s="16">
+        <f>IF(OR(E45="",F45=""),"",MAX(0,7-E45*0.25-F45*0.5))</f>
+        <v/>
+      </c>
       <c r="H45" s="5" t="n"/>
-      <c r="I45" s="6">
+      <c r="I45" s="5">
         <f>IF(COUNTA(A45)=0,"",SUM(B45,C45,D45,E45,F45,G45,H45))</f>
         <v/>
       </c>
-      <c r="J45" s="7">
+      <c r="J45" s="5">
         <f>IF(I45="","",IF(I45&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K45" s="5" t="n"/>
+      <c r="L45" s="5" t="n"/>
+      <c r="M45" s="6">
+        <f>IF(COUNTA(A45)=0,"",IFERROR(SUM(D45,G45,H45,I45,J45,K45,L45),""))</f>
+        <v/>
+      </c>
+      <c r="N45" s="18">
+        <f>IF(M45="","",IF(M45&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1381,17 +2136,33 @@
       <c r="A46" s="8" t="n"/>
       <c r="B46" s="9" t="n"/>
       <c r="C46" s="9" t="n"/>
-      <c r="D46" s="9" t="n"/>
+      <c r="D46" s="16">
+        <f>IF(OR(B46="",C46=""),"",MAX(0,5-B46*0.25-C46*0.5))</f>
+        <v/>
+      </c>
       <c r="E46" s="9" t="n"/>
       <c r="F46" s="9" t="n"/>
-      <c r="G46" s="9" t="n"/>
+      <c r="G46" s="16">
+        <f>IF(OR(E46="",F46=""),"",MAX(0,7-E46*0.25-F46*0.5))</f>
+        <v/>
+      </c>
       <c r="H46" s="9" t="n"/>
-      <c r="I46" s="6">
+      <c r="I46" s="9">
         <f>IF(COUNTA(A46)=0,"",SUM(B46,C46,D46,E46,F46,G46,H46))</f>
         <v/>
       </c>
-      <c r="J46" s="7">
+      <c r="J46" s="9">
         <f>IF(I46="","",IF(I46&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K46" s="9" t="n"/>
+      <c r="L46" s="9" t="n"/>
+      <c r="M46" s="6">
+        <f>IF(COUNTA(A46)=0,"",IFERROR(SUM(D46,G46,H46,I46,J46,K46,L46),""))</f>
+        <v/>
+      </c>
+      <c r="N46" s="17">
+        <f>IF(M46="","",IF(M46&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1399,17 +2170,33 @@
       <c r="A47" s="4" t="n"/>
       <c r="B47" s="5" t="n"/>
       <c r="C47" s="5" t="n"/>
-      <c r="D47" s="5" t="n"/>
+      <c r="D47" s="16">
+        <f>IF(OR(B47="",C47=""),"",MAX(0,5-B47*0.25-C47*0.5))</f>
+        <v/>
+      </c>
       <c r="E47" s="5" t="n"/>
       <c r="F47" s="5" t="n"/>
-      <c r="G47" s="5" t="n"/>
+      <c r="G47" s="16">
+        <f>IF(OR(E47="",F47=""),"",MAX(0,7-E47*0.25-F47*0.5))</f>
+        <v/>
+      </c>
       <c r="H47" s="5" t="n"/>
-      <c r="I47" s="6">
+      <c r="I47" s="5">
         <f>IF(COUNTA(A47)=0,"",SUM(B47,C47,D47,E47,F47,G47,H47))</f>
         <v/>
       </c>
-      <c r="J47" s="7">
+      <c r="J47" s="5">
         <f>IF(I47="","",IF(I47&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K47" s="5" t="n"/>
+      <c r="L47" s="5" t="n"/>
+      <c r="M47" s="6">
+        <f>IF(COUNTA(A47)=0,"",IFERROR(SUM(D47,G47,H47,I47,J47,K47,L47),""))</f>
+        <v/>
+      </c>
+      <c r="N47" s="18">
+        <f>IF(M47="","",IF(M47&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1417,17 +2204,33 @@
       <c r="A48" s="8" t="n"/>
       <c r="B48" s="9" t="n"/>
       <c r="C48" s="9" t="n"/>
-      <c r="D48" s="9" t="n"/>
+      <c r="D48" s="16">
+        <f>IF(OR(B48="",C48=""),"",MAX(0,5-B48*0.25-C48*0.5))</f>
+        <v/>
+      </c>
       <c r="E48" s="9" t="n"/>
       <c r="F48" s="9" t="n"/>
-      <c r="G48" s="9" t="n"/>
+      <c r="G48" s="16">
+        <f>IF(OR(E48="",F48=""),"",MAX(0,7-E48*0.25-F48*0.5))</f>
+        <v/>
+      </c>
       <c r="H48" s="9" t="n"/>
-      <c r="I48" s="6">
+      <c r="I48" s="9">
         <f>IF(COUNTA(A48)=0,"",SUM(B48,C48,D48,E48,F48,G48,H48))</f>
         <v/>
       </c>
-      <c r="J48" s="7">
+      <c r="J48" s="9">
         <f>IF(I48="","",IF(I48&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K48" s="9" t="n"/>
+      <c r="L48" s="9" t="n"/>
+      <c r="M48" s="6">
+        <f>IF(COUNTA(A48)=0,"",IFERROR(SUM(D48,G48,H48,I48,J48,K48,L48),""))</f>
+        <v/>
+      </c>
+      <c r="N48" s="17">
+        <f>IF(M48="","",IF(M48&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1435,17 +2238,33 @@
       <c r="A49" s="4" t="n"/>
       <c r="B49" s="5" t="n"/>
       <c r="C49" s="5" t="n"/>
-      <c r="D49" s="5" t="n"/>
+      <c r="D49" s="16">
+        <f>IF(OR(B49="",C49=""),"",MAX(0,5-B49*0.25-C49*0.5))</f>
+        <v/>
+      </c>
       <c r="E49" s="5" t="n"/>
       <c r="F49" s="5" t="n"/>
-      <c r="G49" s="5" t="n"/>
+      <c r="G49" s="16">
+        <f>IF(OR(E49="",F49=""),"",MAX(0,7-E49*0.25-F49*0.5))</f>
+        <v/>
+      </c>
       <c r="H49" s="5" t="n"/>
-      <c r="I49" s="6">
+      <c r="I49" s="5">
         <f>IF(COUNTA(A49)=0,"",SUM(B49,C49,D49,E49,F49,G49,H49))</f>
         <v/>
       </c>
-      <c r="J49" s="7">
+      <c r="J49" s="5">
         <f>IF(I49="","",IF(I49&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K49" s="5" t="n"/>
+      <c r="L49" s="5" t="n"/>
+      <c r="M49" s="6">
+        <f>IF(COUNTA(A49)=0,"",IFERROR(SUM(D49,G49,H49,I49,J49,K49,L49),""))</f>
+        <v/>
+      </c>
+      <c r="N49" s="18">
+        <f>IF(M49="","",IF(M49&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1453,17 +2272,33 @@
       <c r="A50" s="8" t="n"/>
       <c r="B50" s="9" t="n"/>
       <c r="C50" s="9" t="n"/>
-      <c r="D50" s="9" t="n"/>
+      <c r="D50" s="16">
+        <f>IF(OR(B50="",C50=""),"",MAX(0,5-B50*0.25-C50*0.5))</f>
+        <v/>
+      </c>
       <c r="E50" s="9" t="n"/>
       <c r="F50" s="9" t="n"/>
-      <c r="G50" s="9" t="n"/>
+      <c r="G50" s="16">
+        <f>IF(OR(E50="",F50=""),"",MAX(0,7-E50*0.25-F50*0.5))</f>
+        <v/>
+      </c>
       <c r="H50" s="9" t="n"/>
-      <c r="I50" s="6">
+      <c r="I50" s="9">
         <f>IF(COUNTA(A50)=0,"",SUM(B50,C50,D50,E50,F50,G50,H50))</f>
         <v/>
       </c>
-      <c r="J50" s="7">
+      <c r="J50" s="9">
         <f>IF(I50="","",IF(I50&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K50" s="9" t="n"/>
+      <c r="L50" s="9" t="n"/>
+      <c r="M50" s="6">
+        <f>IF(COUNTA(A50)=0,"",IFERROR(SUM(D50,G50,H50,I50,J50,K50,L50),""))</f>
+        <v/>
+      </c>
+      <c r="N50" s="17">
+        <f>IF(M50="","",IF(M50&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1471,17 +2306,33 @@
       <c r="A51" s="4" t="n"/>
       <c r="B51" s="5" t="n"/>
       <c r="C51" s="5" t="n"/>
-      <c r="D51" s="5" t="n"/>
+      <c r="D51" s="16">
+        <f>IF(OR(B51="",C51=""),"",MAX(0,5-B51*0.25-C51*0.5))</f>
+        <v/>
+      </c>
       <c r="E51" s="5" t="n"/>
       <c r="F51" s="5" t="n"/>
-      <c r="G51" s="5" t="n"/>
+      <c r="G51" s="16">
+        <f>IF(OR(E51="",F51=""),"",MAX(0,7-E51*0.25-F51*0.5))</f>
+        <v/>
+      </c>
       <c r="H51" s="5" t="n"/>
-      <c r="I51" s="6">
+      <c r="I51" s="5">
         <f>IF(COUNTA(A51)=0,"",SUM(B51,C51,D51,E51,F51,G51,H51))</f>
         <v/>
       </c>
-      <c r="J51" s="7">
+      <c r="J51" s="5">
         <f>IF(I51="","",IF(I51&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K51" s="5" t="n"/>
+      <c r="L51" s="5" t="n"/>
+      <c r="M51" s="6">
+        <f>IF(COUNTA(A51)=0,"",IFERROR(SUM(D51,G51,H51,I51,J51,K51,L51),""))</f>
+        <v/>
+      </c>
+      <c r="N51" s="18">
+        <f>IF(M51="","",IF(M51&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1489,17 +2340,33 @@
       <c r="A52" s="8" t="n"/>
       <c r="B52" s="9" t="n"/>
       <c r="C52" s="9" t="n"/>
-      <c r="D52" s="9" t="n"/>
+      <c r="D52" s="16">
+        <f>IF(OR(B52="",C52=""),"",MAX(0,5-B52*0.25-C52*0.5))</f>
+        <v/>
+      </c>
       <c r="E52" s="9" t="n"/>
       <c r="F52" s="9" t="n"/>
-      <c r="G52" s="9" t="n"/>
+      <c r="G52" s="16">
+        <f>IF(OR(E52="",F52=""),"",MAX(0,7-E52*0.25-F52*0.5))</f>
+        <v/>
+      </c>
       <c r="H52" s="9" t="n"/>
-      <c r="I52" s="6">
+      <c r="I52" s="9">
         <f>IF(COUNTA(A52)=0,"",SUM(B52,C52,D52,E52,F52,G52,H52))</f>
         <v/>
       </c>
-      <c r="J52" s="7">
+      <c r="J52" s="9">
         <f>IF(I52="","",IF(I52&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K52" s="9" t="n"/>
+      <c r="L52" s="9" t="n"/>
+      <c r="M52" s="6">
+        <f>IF(COUNTA(A52)=0,"",IFERROR(SUM(D52,G52,H52,I52,J52,K52,L52),""))</f>
+        <v/>
+      </c>
+      <c r="N52" s="17">
+        <f>IF(M52="","",IF(M52&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1507,17 +2374,33 @@
       <c r="A53" s="4" t="n"/>
       <c r="B53" s="5" t="n"/>
       <c r="C53" s="5" t="n"/>
-      <c r="D53" s="5" t="n"/>
+      <c r="D53" s="16">
+        <f>IF(OR(B53="",C53=""),"",MAX(0,5-B53*0.25-C53*0.5))</f>
+        <v/>
+      </c>
       <c r="E53" s="5" t="n"/>
       <c r="F53" s="5" t="n"/>
-      <c r="G53" s="5" t="n"/>
+      <c r="G53" s="16">
+        <f>IF(OR(E53="",F53=""),"",MAX(0,7-E53*0.25-F53*0.5))</f>
+        <v/>
+      </c>
       <c r="H53" s="5" t="n"/>
-      <c r="I53" s="6">
+      <c r="I53" s="5">
         <f>IF(COUNTA(A53)=0,"",SUM(B53,C53,D53,E53,F53,G53,H53))</f>
         <v/>
       </c>
-      <c r="J53" s="7">
+      <c r="J53" s="5">
         <f>IF(I53="","",IF(I53&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K53" s="5" t="n"/>
+      <c r="L53" s="5" t="n"/>
+      <c r="M53" s="6">
+        <f>IF(COUNTA(A53)=0,"",IFERROR(SUM(D53,G53,H53,I53,J53,K53,L53),""))</f>
+        <v/>
+      </c>
+      <c r="N53" s="18">
+        <f>IF(M53="","",IF(M53&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1525,17 +2408,61 @@
       <c r="A54" s="8" t="n"/>
       <c r="B54" s="9" t="n"/>
       <c r="C54" s="9" t="n"/>
-      <c r="D54" s="9" t="n"/>
+      <c r="D54" s="16">
+        <f>IF(OR(B54="",C54=""),"",MAX(0,5-B54*0.25-C54*0.5))</f>
+        <v/>
+      </c>
       <c r="E54" s="9" t="n"/>
       <c r="F54" s="9" t="n"/>
-      <c r="G54" s="9" t="n"/>
+      <c r="G54" s="16">
+        <f>IF(OR(E54="",F54=""),"",MAX(0,7-E54*0.25-F54*0.5))</f>
+        <v/>
+      </c>
       <c r="H54" s="9" t="n"/>
-      <c r="I54" s="6">
+      <c r="I54" s="9">
         <f>IF(COUNTA(A54)=0,"",SUM(B54,C54,D54,E54,F54,G54,H54))</f>
         <v/>
       </c>
-      <c r="J54" s="7">
+      <c r="J54" s="9">
         <f>IF(I54="","",IF(I54&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+      <c r="K54" s="9" t="n"/>
+      <c r="L54" s="9" t="n"/>
+      <c r="M54" s="6">
+        <f>IF(COUNTA(A54)=0,"",IFERROR(SUM(D54,G54,H54,I54,J54,K54,L54),""))</f>
+        <v/>
+      </c>
+      <c r="N54" s="17">
+        <f>IF(M54="","",IF(M54&gt;=30,"✓ Admis","✗ Refusé"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="4" t="n"/>
+      <c r="B55" s="5" t="n"/>
+      <c r="C55" s="5" t="n"/>
+      <c r="D55" s="16">
+        <f>IF(OR(B55="",C55=""),"",MAX(0,5-B55*0.25-C55*0.5))</f>
+        <v/>
+      </c>
+      <c r="E55" s="5" t="n"/>
+      <c r="F55" s="5" t="n"/>
+      <c r="G55" s="16">
+        <f>IF(OR(E55="",F55=""),"",MAX(0,7-E55*0.25-F55*0.5))</f>
+        <v/>
+      </c>
+      <c r="H55" s="5" t="n"/>
+      <c r="I55" s="5" t="n"/>
+      <c r="J55" s="5" t="n"/>
+      <c r="K55" s="5" t="n"/>
+      <c r="L55" s="5" t="n"/>
+      <c r="M55" s="6">
+        <f>IF(COUNTA(A55)=0,"",IFERROR(SUM(D55,G55,H55,I55,J55,K55,L55),""))</f>
+        <v/>
+      </c>
+      <c r="N55" s="18">
+        <f>IF(M55="","",IF(M55&gt;=30,"✓ Admis","✗ Refusé"))</f>
         <v/>
       </c>
     </row>
@@ -1547,10 +2474,14 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="7">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A56:J56"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="E4:G4"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>